<commit_message>
fix: cldf normaliza nome maiúsculo e documenta descarte de linha sem data
- Normaliza nomes em CAIXA ALTA (formato pivô) para Title Case em _politico()
- Envolve parse() em try/finally para garantir fechamento de workbook
- Adiciona comentário explicando descarte de linha sem data em _parse_transacional
- Adiciona linha sem data às fixtures para cobrir caso descartado
- Adiciona testes: test_pivo_normaliza_nome_maiusculo e test_transacional_linha_sem_data_e_ignorada

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/cldf_transacional.xlsx
+++ b/backend/tests/fixtures/cldf_transacional.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -583,6 +583,31 @@
         <is>
           <t>Locação de imóvel</t>
         </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Deputado Chico Vigilante</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FORNECEDOR SEM DATA</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: cldf tolera formatos reais (colunas 2013, valores/datas string BR)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/cldf_transacional.xlsx
+++ b/backend/tests/fixtures/cldf_transacional.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -608,6 +608,126 @@
       </c>
       <c r="H5" t="n">
         <v>999</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Deputada Jane Klebia</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>HOTEL XYZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>03.333.333/0003-33</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>42500</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>R$ 5.000,00</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Hospedagem</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Deputado Chico Vigilante</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TRANSPORTADORA ABC</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>04.444.444/0004-44</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>42536</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>9,900,00</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Locação de veículos</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Deputada Jane Klebia</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>RESTAURANTE DEF</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>555.666.777-88</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>15/05/2016</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>700</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>